<commit_message>
Update Nalco PDF (2026-03-04 05:33:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -19,16 +19,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,24 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -436,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -448,760 +433,788 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sl.no.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Product Code</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Basic Price</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Circular Date</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Circular Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>339.45</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>01-03-2026</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>330.75</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>14-01-2026</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>320.05</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>07-01-2026</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
+    <row r="5">
+      <c r="A5" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>307.25</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>01-01-2026</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>301.65</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>24-12-2025</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
+    <row r="7">
+      <c r="A7" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>296.05</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>05-12-2025</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
+    <row r="8">
+      <c r="A8" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>290.95</v>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>27-11-2025</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
         <v>283.55</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>22-11-2025</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
+    <row r="10">
+      <c r="A10" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
         <v>281.95</v>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>19-11-2025</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
         <v>292.65</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>07-11-2025</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
+    <row r="12">
+      <c r="A12" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
         <v>296.05</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>02-11-2025</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="n">
+    <row r="13">
+      <c r="A13" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
         <v>297.15</v>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>01-11-2025</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
+    <row r="14">
+      <c r="A14" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
         <v>294.05</v>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>30-10-2025</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
+    <row r="15">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
         <v>288.55</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>25-10-2025</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
+    <row r="16">
+      <c r="A16" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
         <v>282.45</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>17-10-2025</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
+    <row r="17">
+      <c r="A17" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
         <v>285.05</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>14-10-2025</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>282.85</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>09-10-2025</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
+    <row r="19">
+      <c r="A19" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
         <v>277.95</v>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>01-10-2025</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
         <v>274.95</v>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>30-09-2025</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
+    <row r="21">
+      <c r="A21" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
         <v>270.25</v>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>25-09-2025</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
+    <row r="22">
+      <c r="A22" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
         <v>275.25</v>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>20-09-2025</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
+    <row r="23">
+      <c r="A23" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
         <v>278.95</v>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>17-09-2025</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
+    <row r="24">
+      <c r="A24" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
         <v>272.05</v>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>01-09-2025</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="n">
+    <row r="25">
+      <c r="A25" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n">
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
         <v>271.05</v>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>28-08-2025</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
+    <row r="26">
+      <c r="A26" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
         <v>264.35</v>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>21-08-2025</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="n">
+    <row r="27">
+      <c r="A27" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
         <v>269.45</v>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>15-08-2025</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
+    <row r="28">
+      <c r="A28" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="n">
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1235,6 +1248,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-04 06:37:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -494,7 +494,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>330.75</v>
+        <v>330.95</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>320.05</v>
+        <v>323.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>307.25</v>
+        <v>318.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>301.65</v>
+        <v>320.45</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>296.05</v>
+        <v>316.15</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>290.95</v>
+        <v>330.75</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>283.55</v>
+        <v>323.75</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>281.95</v>
+        <v>320.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>292.65</v>
+        <v>307.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>294.05</v>
+        <v>290.95</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>288.55</v>
+        <v>283.55</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>282.45</v>
+        <v>281.95</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>285.05</v>
+        <v>292.65</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>282.85</v>
+        <v>296.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>277.95</v>
+        <v>297.15</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>274.95</v>
+        <v>294.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>270.25</v>
+        <v>288.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>275.25</v>
+        <v>282.45</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>278.95</v>
+        <v>285.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>272.05</v>
+        <v>282.85</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>271.05</v>
+        <v>277.95</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>264.35</v>
+        <v>274.95</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,42 +1179,210 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>269.45</v>
+        <v>270.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>275.25</v>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>20-09-2025</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>278.95</v>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>17-09-2025</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>01-09-2025</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>271.05</v>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>28-08-2025</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>264.35</v>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>21-08-2025</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="n">
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1249,6 +1417,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-04 06:56:06 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -550,7 +550,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>318.05</v>
+        <v>316.15</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>320.45</v>
+        <v>323.75</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>316.15</v>
+        <v>318.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>330.75</v>
+        <v>320.45</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>323.75</v>
+        <v>333.45</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>320.05</v>
+        <v>325.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>307.25</v>
+        <v>316.15</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>301.65</v>
+        <v>330.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>296.05</v>
+        <v>323.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>290.95</v>
+        <v>320.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>283.55</v>
+        <v>307.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>281.95</v>
+        <v>301.65</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>292.65</v>
+        <v>296.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>296.05</v>
+        <v>290.95</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>297.15</v>
+        <v>283.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>294.05</v>
+        <v>281.95</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>288.55</v>
+        <v>292.65</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>282.45</v>
+        <v>296.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>285.05</v>
+        <v>297.15</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>282.85</v>
+        <v>294.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>277.95</v>
+        <v>288.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>274.95</v>
+        <v>282.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>270.25</v>
+        <v>285.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>275.25</v>
+        <v>282.85</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>278.95</v>
+        <v>277.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>272.05</v>
+        <v>274.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>271.05</v>
+        <v>270.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>264.35</v>
+        <v>275.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,42 +1347,154 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>269.45</v>
+        <v>278.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>272.05</v>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>01-09-2025</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>271.05</v>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>28-08-2025</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>264.35</v>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>21-08-2025</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="n">
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E38" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F38" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1423,6 +1535,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-06 04:54:37 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,42 +1403,70 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B36" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C36" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="n">
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E37" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1481,6 +1509,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-11 04:56:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,42 +1431,70 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B37" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C37" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="n">
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E37" s="1" t="inlineStr">
+      <c r="E38" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F37" s="1" t="inlineStr">
+      <c r="F38" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1510,6 +1538,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-14 04:56:16 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,42 +1459,70 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B38" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C38" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="n">
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E38" s="1" t="inlineStr">
+      <c r="E39" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F38" s="1" t="inlineStr">
+      <c r="F39" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1539,6 +1567,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-19 05:08:57 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,42 +1487,70 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C39" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="n">
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E39" s="1" t="inlineStr">
+      <c r="E40" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F39" s="1" t="inlineStr">
+      <c r="F40" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1568,6 +1596,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-24 05:09:39 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,42 +1515,70 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B40" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C40" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="n">
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E40" s="1" t="inlineStr">
+      <c r="E41" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F40" s="1" t="inlineStr">
+      <c r="F41" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1597,6 +1625,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-03-28 05:08:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,42 +1543,70 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B41" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C41" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="n">
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E41" s="1" t="inlineStr">
+      <c r="E42" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F41" s="1" t="inlineStr">
+      <c r="F42" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1626,6 +1654,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-04-03 05:19:18 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,42 +1571,70 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C42" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="n">
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E42" s="1" t="inlineStr">
+      <c r="E43" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F42" s="1" t="inlineStr">
+      <c r="F43" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1655,6 +1683,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-04-16 05:40:39 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,42 +1599,70 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="n">
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E43" s="1" t="inlineStr">
+      <c r="E44" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F43" s="1" t="inlineStr">
+      <c r="F44" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1684,6 +1712,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-04-24 05:53:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,42 +1627,70 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C44" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="n">
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E44" s="1" t="inlineStr">
+      <c r="E45" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F44" s="1" t="inlineStr">
+      <c r="F45" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1713,6 +1741,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-05-05 06:00:58 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,42 +1655,70 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C45" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="n">
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E45" s="1" t="inlineStr">
+      <c r="E46" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F45" s="1" t="inlineStr">
+      <c r="F46" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1742,6 +1770,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-05-14 06:35:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,42 +1683,70 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="n">
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E46" s="1" t="inlineStr">
+      <c r="E47" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F46" s="1" t="inlineStr">
+      <c r="F47" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1771,6 +1799,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-05-20 06:59:28 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,42 +1711,70 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B47" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C47" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="n">
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E47" s="1" t="inlineStr">
+      <c r="E48" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F47" s="1" t="inlineStr">
+      <c r="F48" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1800,6 +1828,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-05-27 07:46:07 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,42 +1739,70 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="n">
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E48" s="1" t="inlineStr">
+      <c r="E49" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F48" s="1" t="inlineStr">
+      <c r="F49" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1829,6 +1857,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-02 08:11:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,42 +1767,70 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C49" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="n">
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E49" s="1" t="inlineStr">
+      <c r="E50" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F49" s="1" t="inlineStr">
+      <c r="F50" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1858,6 +1886,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-05 07:50:02 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,42 +1795,70 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C50" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="n">
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E50" s="1" t="inlineStr">
+      <c r="E51" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F50" s="1" t="inlineStr">
+      <c r="F51" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1887,6 +1915,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-10 07:50:44 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,42 +1823,70 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C51" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="n">
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E51" s="1" t="inlineStr">
+      <c r="E52" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F51" s="1" t="inlineStr">
+      <c r="F52" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1916,6 +1944,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-13 07:08:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,42 +1851,70 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C52" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="n">
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E52" s="1" t="inlineStr">
+      <c r="E53" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F52" s="1" t="inlineStr">
+      <c r="F53" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1945,6 +1973,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-18 08:22:38 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,42 +1879,70 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="n">
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E53" s="1" t="inlineStr">
+      <c r="E54" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F53" s="1" t="inlineStr">
+      <c r="F54" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -1974,6 +2002,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-26 07:06:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,42 +1907,70 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C54" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="n">
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E54" s="1" t="inlineStr">
+      <c r="E55" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F54" s="1" t="inlineStr">
+      <c r="F55" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2003,6 +2031,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-26 11:57:42 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,42 +1935,70 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C55" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="n">
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E55" s="1" t="inlineStr">
+      <c r="E56" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F55" s="1" t="inlineStr">
+      <c r="F56" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2032,6 +2060,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-06-29 08:30:17 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -483,18 +483,18 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,42 +1963,70 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C56" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="n">
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E56" s="1" t="inlineStr">
+      <c r="E57" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F56" s="1" t="inlineStr">
+      <c r="F57" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2061,6 +2089,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-02 06:53:13 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -511,18 +511,18 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,42 +1991,70 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B57" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C57" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="n">
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E57" s="1" t="inlineStr">
+      <c r="E58" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F57" s="1" t="inlineStr">
+      <c r="F58" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2090,6 +2118,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-08 06:10:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -539,18 +539,18 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,42 +2019,70 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B58" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C58" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="n">
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E58" s="1" t="inlineStr">
+      <c r="E59" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F58" s="1" t="inlineStr">
+      <c r="F59" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2119,6 +2147,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-13 06:36:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -567,18 +567,18 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,42 +2047,70 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B59" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C59" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="n">
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E59" s="1" t="inlineStr">
+      <c r="E60" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F59" s="1" t="inlineStr">
+      <c r="F60" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2148,6 +2176,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-18 05:40:47 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -595,18 +595,18 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,42 +2075,70 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B60" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C60" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="n">
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E60" s="1" t="inlineStr">
+      <c r="E61" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F60" s="1" t="inlineStr">
+      <c r="F61" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2177,6 +2205,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-24 06:07:39 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -623,18 +623,18 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,42 +2103,70 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="n">
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E61" s="1" t="inlineStr">
+      <c r="E62" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F61" s="1" t="inlineStr">
+      <c r="F62" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2206,6 +2234,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-07-29 06:12:18 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -651,18 +651,18 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,42 +2131,70 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="n">
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E62" s="1" t="inlineStr">
+      <c r="E63" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F62" s="1" t="inlineStr">
+      <c r="F63" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2235,6 +2263,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-08-04 06:08:23 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -679,18 +679,18 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,42 +2159,70 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="n">
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E63" s="1" t="inlineStr">
+      <c r="E64" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F63" s="1" t="inlineStr">
+      <c r="F64" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2264,6 +2292,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-08-12 05:12:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -707,18 +707,18 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -774,7 +774,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,42 +2187,70 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B64" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="n">
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E64" s="1" t="inlineStr">
+      <c r="E65" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F64" s="1" t="inlineStr">
+      <c r="F65" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2293,6 +2321,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-08-17 07:29:37 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -735,18 +735,18 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -802,7 +802,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,42 +2215,70 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F65" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B65" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="n">
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E65" s="1" t="inlineStr">
+      <c r="E66" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F65" s="1" t="inlineStr">
+      <c r="F66" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2322,6 +2350,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-08-21 07:21:52 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -763,18 +763,18 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,42 +2243,70 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F66" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B66" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C66" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="n">
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E66" s="1" t="inlineStr">
+      <c r="E67" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F66" s="1" t="inlineStr">
+      <c r="F67" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2351,6 +2379,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-08-28 15:32:37 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -791,18 +791,18 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -871,22 +871,22 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,42 +2271,70 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F67" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C67" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="n">
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E67" s="1" t="inlineStr">
+      <c r="E68" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F67" s="1" t="inlineStr">
+      <c r="F68" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2380,6 +2408,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco PDF (2026-09-02 08:01:35 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_prices.xlsx
+++ b/data/nalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -479,22 +479,22 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>360.15</v>
+        <v>361.65</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
@@ -507,22 +507,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>356.25</v>
+        <v>360.15</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>21-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>362.35</v>
+        <v>356.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-21-08-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
@@ -563,22 +563,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>375.25</v>
+        <v>362.35</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-15-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -591,22 +591,22 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>363.35</v>
+        <v>375.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>12-08-2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-12-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -619,22 +619,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>354.95</v>
+        <v>363.35</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-08-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
@@ -647,22 +647,22 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>361.15</v>
+        <v>354.95</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>356.35</v>
+        <v>361.15</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>352.85</v>
+        <v>356.35</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
@@ -731,22 +731,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>349.05</v>
+        <v>352.85</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>11-07-2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
@@ -759,22 +759,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>344.05</v>
+        <v>349.05</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-08-07-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>349.05</v>
+        <v>344.05</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-07-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
@@ -819,18 +819,18 @@
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>26-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
@@ -843,22 +843,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>376.55</v>
+        <v>349.05</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-26-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
@@ -899,22 +899,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>393.85</v>
+        <v>376.55</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
@@ -927,22 +927,22 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>402.35</v>
+        <v>393.85</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>10-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
@@ -955,22 +955,22 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>416.35</v>
+        <v>402.35</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>05-06-2026</t>
+          <t>10-06-2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-10-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>412.55</v>
+        <v>416.35</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
@@ -1011,22 +1011,22 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>411.05</v>
+        <v>412.55</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>27-05-2026</t>
+          <t>01-06-2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-06-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>404.95</v>
+        <v>411.05</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>20-05-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
@@ -1067,22 +1067,22 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>408.85</v>
+        <v>404.95</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-20-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
@@ -1095,22 +1095,22 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>390.05</v>
+        <v>408.85</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>392.55</v>
+        <v>390.05</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-05-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
@@ -1151,22 +1151,22 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>383.65</v>
+        <v>392.55</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>16-04-2026</t>
+          <t>24-04-2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
@@ -1179,22 +1179,22 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>373.55</v>
+        <v>383.65</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>16-04-2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-04-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
@@ -1207,22 +1207,22 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>357.05</v>
+        <v>373.55</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>03-04-2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-04-26.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>350.45</v>
+        <v>357.05</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>28-03-2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
@@ -1263,22 +1263,22 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>360.05</v>
+        <v>350.45</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>19-03-2026</t>
+          <t>24-03-2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>372.05</v>
+        <v>360.05</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>14-03-2026</t>
+          <t>19-03-2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
@@ -1319,22 +1319,22 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>358.75</v>
+        <v>372.05</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>11-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot14.03.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
@@ -1347,22 +1347,22 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>347.25</v>
+        <v>358.75</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>06-03-2026</t>
+          <t>11-03-2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
@@ -1375,22 +1375,22 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>339.45</v>
+        <v>347.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>06-03-2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-06-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
@@ -1403,22 +1403,22 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>330.95</v>
+        <v>339.45</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-03-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>323.05</v>
+        <v>330.95</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
@@ -1459,22 +1459,22 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>316.15</v>
+        <v>323.05</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-02-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>323.75</v>
+        <v>316.15</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-18-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
@@ -1515,22 +1515,22 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>318.05</v>
+        <v>323.75</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-12-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>320.45</v>
+        <v>318.05</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>333.45</v>
+        <v>320.45</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-02-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
@@ -1599,22 +1599,22 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>325.35</v>
+        <v>333.45</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-28-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
@@ -1627,22 +1627,22 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>330.75</v>
+        <v>325.35</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-23.01.2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
@@ -1655,22 +1655,22 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>320.05</v>
+        <v>330.75</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
@@ -1683,22 +1683,22 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>307.25</v>
+        <v>320.05</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/01/Ingot-07-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
@@ -1711,22 +1711,22 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>301.65</v>
+        <v>307.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-01-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
@@ -1739,22 +1739,22 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>296.05</v>
+        <v>301.65</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
@@ -1767,22 +1767,22 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>290.95</v>
+        <v>296.05</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-05-12-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
@@ -1795,22 +1795,22 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>283.55</v>
+        <v>290.95</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-27-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
@@ -1823,22 +1823,22 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>281.95</v>
+        <v>283.55</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/11/Ingot-22-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>292.65</v>
+        <v>281.95</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
@@ -1879,22 +1879,22 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>296.05</v>
+        <v>292.65</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
@@ -1907,22 +1907,22 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>297.15</v>
+        <v>296.05</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-02-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
@@ -1935,22 +1935,22 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>294.05</v>
+        <v>297.15</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-11-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>288.55</v>
+        <v>294.05</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-30-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
@@ -1991,22 +1991,22 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>282.45</v>
+        <v>288.55</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-25-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
@@ -2019,22 +2019,22 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>285.05</v>
+        <v>282.45</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-17-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
@@ -2047,22 +2047,22 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>282.85</v>
+        <v>285.05</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-14-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
@@ -2075,22 +2075,22 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>277.95</v>
+        <v>282.85</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-09-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>274.95</v>
+        <v>277.95</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
@@ -2131,22 +2131,22 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>270.25</v>
+        <v>274.95</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/09/INGOT-30-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
@@ -2159,22 +2159,22 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>275.25</v>
+        <v>270.25</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-25-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
@@ -2187,22 +2187,22 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>278.95</v>
+        <v>275.25</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-20-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
@@ -2215,22 +2215,22 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>272.05</v>
+        <v>278.95</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-17-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
@@ -2243,22 +2243,22 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>271.05</v>
+        <v>272.05</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-01-09-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>264.35</v>
+        <v>271.05</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-28-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
@@ -2299,42 +2299,70 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>269.45</v>
+        <v>264.35</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/INGOT-21-08-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C68" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="E68" s="1" t="inlineStr">
+        <is>
+          <t>15-08-2025</t>
+        </is>
+      </c>
+      <c r="F68" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2025/08/INGOT-15-08-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B68" s="1" t="inlineStr">
-        <is>
-          <t>ALUMINIUM INGOT</t>
-        </is>
-      </c>
-      <c r="C68" s="1" t="inlineStr">
-        <is>
-          <t>IE07</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="n">
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>ALUMINIUM INGOT</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>IE07</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
         <v>268.25</v>
       </c>
-      <c r="E68" s="1" t="inlineStr">
+      <c r="E69" s="1" t="inlineStr">
         <is>
           <t>07-08-2025</t>
         </is>
       </c>
-      <c r="F68" s="1" t="inlineStr">
+      <c r="F69" s="1" t="inlineStr">
         <is>
           <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-07-08-2025.pdf</t>
         </is>
@@ -2409,6 +2437,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>